<commit_message>
chore: sync latest entries from dictionary_entries.xlsx to CSV
</commit_message>
<xml_diff>
--- a/data/i18n/dictionary_entries.xlsx
+++ b/data/i18n/dictionary_entries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yezi\G_project\S2_mission_game\fukuchange_v2\data\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7C878AE-A319-4CA9-8A28-997C84AC2C7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{666594E2-1445-4BA2-90C9-8AD626C93CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-45" yWindow="315" windowWidth="24420" windowHeight="15150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="7815" windowWidth="17610" windowHeight="7650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="詞典資料" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">詞典資料!$A$1:$U$21</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -331,7 +330,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="283">
   <si>
     <t>啟用</t>
   </si>
@@ -417,9 +416,6 @@
     <t>透氣清爽的短袖棉質上衣，適合夏日活動。</t>
   </si>
   <si>
-    <t>donˋ qiu</t>
-  </si>
-  <si>
     <t>V</t>
   </si>
   <si>
@@ -435,9 +431,6 @@
     <t>長褲</t>
   </si>
   <si>
-    <t>適合在郊外穿，能遮擋蚊蟲。</t>
-  </si>
-  <si>
     <t>30</t>
   </si>
   <si>
@@ -648,9 +641,6 @@
     <t>#f97316</t>
   </si>
   <si>
-    <t>橘色</t>
-  </si>
-  <si>
     <t>gamˊ eˋ sedˋ</t>
   </si>
   <si>
@@ -678,9 +668,6 @@
     <t>#ffffff</t>
   </si>
   <si>
-    <t>白色</t>
-  </si>
-  <si>
     <t>pag sedˋ</t>
   </si>
   <si>
@@ -693,9 +680,6 @@
     <t>#1e293b</t>
   </si>
   <si>
-    <t>黑色</t>
-  </si>
-  <si>
     <t>烏色</t>
   </si>
   <si>
@@ -711,9 +695,6 @@
     <t>#542480</t>
   </si>
   <si>
-    <t>紫色</t>
-  </si>
-  <si>
     <t>吊菜色</t>
   </si>
   <si>
@@ -730,12 +711,6 @@
   </si>
   <si>
     <t>#ec4899</t>
-  </si>
-  <si>
-    <t>紅色花布</t>
-  </si>
-  <si>
-    <t>fungˇ sedˋ faˊ bu</t>
   </si>
   <si>
     <t>欄位</t>
@@ -1236,10 +1211,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>短袖</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>gamˊ eˋ sedˋ</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1304,11 +1275,51 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>紅色花布</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>qiuˇ suiˋ samˊ</t>
+    <t>適合在郊外穿，能遮擋蚊蟲。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>橘色，像柑橘一樣鮮豔。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>黃色，是金黃燦爛的杭菊色彩。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>白色，是如雪般潔白的杭菊色彩。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花布，充滿熱情喜慶與傳統風情的花色，</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>黑色，是沉穩低調的經典色彩。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>紫色，是高貴浪漫的迷人色彩。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>qiuˇ siuˋ samˊ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花布色</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>faˊ bu sedˋ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>短袖衫</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>donˋ qiu samˊ</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1800,8 +1811,8 @@
     <col min="5" max="5" width="13.140625" customWidth="1"/>
     <col min="6" max="6" width="4.7109375" customWidth="1"/>
     <col min="7" max="7" width="2.7109375" customWidth="1"/>
-    <col min="8" max="8" width="5.5703125" customWidth="1"/>
-    <col min="9" max="9" width="5.85546875" customWidth="1"/>
+    <col min="8" max="8" width="10.42578125" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" customWidth="1"/>
     <col min="10" max="10" width="8.5703125" customWidth="1"/>
     <col min="11" max="11" width="15.28515625" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
@@ -1906,40 +1917,40 @@
         <v>27</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
       <c r="K2" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="L2" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="10" t="s">
-        <v>29</v>
-      </c>
       <c r="M2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="U2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1950,57 +1961,57 @@
         <v>22</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>31</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>34</v>
+        <v>271</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="U3" s="6" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:21" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2011,55 +2022,55 @@
         <v>22</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="I4" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="J4" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="L4" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="O4" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>221</v>
-      </c>
       <c r="P4" s="6" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="Q4" s="6" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="R4" s="6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
     </row>
     <row r="5" spans="1:21" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2070,173 +2081,173 @@
         <v>22</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="J5" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>46</v>
-      </c>
       <c r="L5" s="6" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:21" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="H6" s="6" t="s">
+      <c r="J6" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>52</v>
-      </c>
       <c r="L6" s="6" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="N6" s="6" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="O6" s="6" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="P6" s="6" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="Q6" s="6" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="S6" s="6" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="T6" s="6" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="U6" s="6" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="H7" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="I7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="J7" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="I7" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>58</v>
-      </c>
       <c r="L7" s="6" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2247,55 +2258,55 @@
         <v>22</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="H8" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="I8" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="J8" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="I8" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>64</v>
-      </c>
       <c r="L8" s="6" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2306,114 +2317,114 @@
         <v>22</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="H9" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="I9" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H9" s="6" t="s">
+      <c r="J9" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="I9" s="6" t="s">
+      <c r="K9" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="J9" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="L9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="M9" s="6" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="N9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="O9" s="6" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="P9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="Q9" s="6" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="S9" s="6" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="T9" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="U9" s="6" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="1:21" s="6" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="L10" s="13" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="M10" s="13" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="N10" s="13" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="O10" s="13" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="P10" s="13" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="Q10" s="13" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="R10" s="13" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="S10" s="13" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="T10" s="13" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="U10" s="13" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2424,55 +2435,55 @@
         <v>22</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="H11" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="I11" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="J11" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="K11" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="I11" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>77</v>
-      </c>
       <c r="L11" s="6" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:21" s="6" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2483,55 +2494,55 @@
         <v>22</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="H12" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="I12" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="6" t="s">
+      <c r="J12" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="I12" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>83</v>
-      </c>
       <c r="L12" s="6" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
     </row>
     <row r="13" spans="1:21" s="6" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2542,55 +2553,55 @@
         <v>22</v>
       </c>
       <c r="C13" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="H13" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="I13" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="H13" s="6" t="s">
+      <c r="J13" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="K13" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="J13" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>90</v>
-      </c>
       <c r="L13" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="14" spans="1:21" s="6" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2601,58 +2612,58 @@
         <v>22</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="H14" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="I14" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="H14" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>95</v>
-      </c>
       <c r="J14" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="K14" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>254</v>
-      </c>
       <c r="L14" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="O14" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="P14" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q14" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="R14" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="S14" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="T14" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="U14" s="6" t="s">
         <v>246</v>
       </c>
-      <c r="M14" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="N14" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="O14" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="P14" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="Q14" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="R14" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="S14" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="T14" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="U14" s="6" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:21" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>21</v>
       </c>
@@ -2660,113 +2671,113 @@
         <v>22</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E15" s="6" t="s">
         <v>96</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>98</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>262</v>
+        <v>254</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="L15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="M15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T15" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="U15" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" s="6" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="H16" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="K16" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="J16" s="6" t="s">
+      <c r="L16" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="P16" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q16" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="R16" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="S16" s="6" t="s">
         <v>261</v>
       </c>
-      <c r="K16" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="O16" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="Q16" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="R16" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="S16" s="6" t="s">
-        <v>270</v>
-      </c>
       <c r="T16" s="6" t="s">
-        <v>261</v>
+        <v>253</v>
       </c>
       <c r="U16" s="6" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
     </row>
     <row r="17" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2774,55 +2785,55 @@
         <v>21</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C17" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="J17" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="K17" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="F17" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>111</v>
-      </c>
       <c r="L17" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18" spans="1:21" s="6" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2830,55 +2841,55 @@
         <v>21</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C18" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="K18" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>116</v>
-      </c>
       <c r="L18" s="6" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="U18" s="6" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="19" spans="1:21" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -2886,174 +2897,174 @@
         <v>21</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C19" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="K19" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="K19" s="6" t="s">
-        <v>122</v>
-      </c>
       <c r="L19" s="6" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>126</v>
+        <v>277</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>259</v>
+        <v>251</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" ht="47.25" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" ht="78.75" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>133</v>
+        <v>275</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="K21" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="K21" s="6" t="s">
-        <v>134</v>
-      </c>
       <c r="L21" s="10" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="M21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="R21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="T21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="U21" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -3085,13 +3096,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3102,7 +3113,7 @@
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3110,10 +3121,10 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C3" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3124,7 +3135,7 @@
         <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3132,10 +3143,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3146,7 +3157,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3154,10 +3165,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -3176,47 +3187,47 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3236,18 +3247,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B2" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3255,7 +3266,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3263,23 +3274,23 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="B5" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: sync dictionary_entries.xlsx to CSV and confirm six-dialect question sentence dynamic mapping
</commit_message>
<xml_diff>
--- a/data/i18n/dictionary_entries.xlsx
+++ b/data/i18n/dictionary_entries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yezi\G_project\S2_mission_game\fukuchange_v2\data\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{666594E2-1445-4BA2-90C9-8AD626C93CCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA24CEA-CFD0-4479-A993-21F2C8C98EF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="7815" windowWidth="17610" windowHeight="7650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1279,10 +1279,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>橘色，像柑橘一樣鮮豔。</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>黃色，是金黃燦爛的杭菊色彩。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1291,10 +1287,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>花布，充滿熱情喜慶與傳統風情的花色，</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>黑色，是沉穩低調的經典色彩。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1320,6 +1312,14 @@
   </si>
   <si>
     <t>donˋ qiu samˊ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>橘色，是溫暖活潑的快樂色彩。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花布，充滿熱情喜慶與傳統風情的花色。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1917,10 +1917,10 @@
         <v>27</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="L2" s="10" t="s">
         <v>28</v>
@@ -2691,7 +2691,7 @@
         <v>254</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>28</v>
@@ -2724,7 +2724,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:21" s="6" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>21</v>
       </c>
@@ -2741,7 +2741,7 @@
         <v>102</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>253</v>
@@ -2797,7 +2797,7 @@
         <v>106</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>107</v>
@@ -2853,7 +2853,7 @@
         <v>111</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>190</v>
@@ -2909,7 +2909,7 @@
         <v>115</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>116</v>
@@ -2965,7 +2965,7 @@
         <v>120</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>201</v>
@@ -3027,14 +3027,14 @@
         <v>21</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="L21" s="10" t="s">
         <v>166</v>

</xml_diff>

<commit_message>
Update hakka_shirt_B.png image and dictionary_entries CSV/XLSX data
</commit_message>
<xml_diff>
--- a/data/i18n/dictionary_entries.xlsx
+++ b/data/i18n/dictionary_entries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yezi\G_project\S2_mission_game\fukuchange_v2\data\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA24CEA-CFD0-4479-A993-21F2C8C98EF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E71FC345-B392-423E-8745-A135C848C6EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="7815" windowWidth="17610" windowHeight="7650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11535" yWindow="210" windowWidth="17205" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="詞典資料" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,18 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">詞典資料!$A$1:$U$21</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -330,7 +341,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="297">
   <si>
     <t>啟用</t>
   </si>
@@ -413,9 +424,6 @@
     <t>短袖上衣</t>
   </si>
   <si>
-    <t>透氣清爽的短袖棉質上衣，適合夏日活動。</t>
-  </si>
-  <si>
     <t>V</t>
   </si>
   <si>
@@ -443,9 +451,6 @@
     <t>短褲</t>
   </si>
   <si>
-    <t>運動與高溫天氣的清涼選擇。</t>
-  </si>
-  <si>
     <t>donˋ fu</t>
   </si>
   <si>
@@ -461,9 +466,6 @@
     <t>裙子</t>
   </si>
   <si>
-    <t>舒適的日常或宴會的優雅打扮。</t>
-  </si>
-  <si>
     <t>kiunˇ</t>
   </si>
   <si>
@@ -497,9 +499,6 @@
     <t>毛衣</t>
   </si>
   <si>
-    <t>針織膨線毛衣，觸感溫暖舒適。</t>
-  </si>
-  <si>
     <t>pong xien samˊ</t>
   </si>
   <si>
@@ -533,9 +532,6 @@
     <t>鞋子</t>
   </si>
   <si>
-    <t>適合健行等活動的運動鞋。</t>
-  </si>
-  <si>
     <t>鞋</t>
   </si>
   <si>
@@ -587,12 +583,6 @@
     <t>hakka_shirt_B.png</t>
   </si>
   <si>
-    <t>客家藍衫</t>
-  </si>
-  <si>
-    <t>傳統客家婦女的經典藍染大襟衫。</t>
-  </si>
-  <si>
     <t>藍衫</t>
   </si>
   <si>
@@ -842,10 +832,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>V</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>heˇ</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -863,10 +849,6 @@
   </si>
   <si>
     <t>水靴筒</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>shuiˊ hioˋ tung</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1215,10 +1197,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>gamˋ er sed</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>柑色</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1239,10 +1217,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>shui^ hio+ tungˇ</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>水鞋笐</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1320,6 +1294,145 @@
   </si>
   <si>
     <t>花布，充滿熱情喜慶與傳統風情的花色。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>短袖衫</t>
+  </si>
+  <si>
+    <r>
+      <t>donˊ ciu</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF9C6500"/>
+        <rFont val="Tahoma"/>
+        <family val="1"/>
+        <charset val="1"/>
+      </rPr>
+      <t>⁺</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF9C6500"/>
+        <rFont val="新細明體"/>
+        <family val="1"/>
+        <charset val="136"/>
+      </rPr>
+      <t xml:space="preserve"> samˋ</t>
+    </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>don^ ciuˋ sam+</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>水靴</t>
+  </si>
+  <si>
+    <t>suiˋ hioˊ tungˇ</t>
+  </si>
+  <si>
+    <t>shuiˊ hioˋ tung</t>
+  </si>
+  <si>
+    <t xml:space="preserve">shui^ hioˊ </t>
+  </si>
+  <si>
+    <t>ciu shuiˊ samˋ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>ciuˇ shiu^ sam+</t>
+  </si>
+  <si>
+    <t>qiuˇ suiˋ samˊ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>柑色</t>
+  </si>
+  <si>
+    <t>gamˋ sed</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花布</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>faˋ buˇ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花色</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">fa+  sed^ </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花布仔</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>faˊ bu eˋ</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>藍衫</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>傳統客家女孩的經典藍染大襟。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>針織毛衣，觸感溫暖舒適。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>透氣清爽的短袖棉質上衣，適合夏日活動。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>運動與高溫天氣的清涼選擇。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>舒適的日常或宴會的優雅打扮</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Microsoft JhengHei UI"/>
+        <family val="2"/>
+        <charset val="136"/>
+      </rPr>
+      <t>，較不防寒</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="新細明體"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>。</t>
+    </r>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>適合健行、外出等活動的鞋子。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1327,7 +1440,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1381,6 +1494,13 @@
       <name val="Tahoma"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Microsoft JhengHei UI"/>
+      <family val="2"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1464,7 +1584,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1497,6 +1617,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1816,7 +1939,7 @@
     <col min="10" max="10" width="8.5703125" customWidth="1"/>
     <col min="11" max="11" width="15.28515625" customWidth="1"/>
     <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="13" max="13" width="17.28515625" customWidth="1"/>
     <col min="14" max="14" width="14" customWidth="1"/>
     <col min="15" max="15" width="16" customWidth="1"/>
     <col min="16" max="16" width="10.140625" customWidth="1"/>
@@ -1914,43 +2037,43 @@
         <v>26</v>
       </c>
       <c r="I2" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>269</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="M2" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="P2" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="J2" s="6" t="s">
-        <v>279</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>280</v>
-      </c>
-      <c r="L2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="M2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="N2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="O2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="P2" s="10" t="s">
-        <v>28</v>
-      </c>
       <c r="Q2" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R2" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="T2" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="U2" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="T2" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="U2" s="6" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1961,57 +2084,57 @@
         <v>22</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="K3" s="6" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="L3" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="N3" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="O3" s="6" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="T3" s="6" t="s">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="U3" s="6" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:21" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2022,58 +2145,58 @@
         <v>22</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="6" t="s">
+      <c r="I4" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="K4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="J4" s="6" t="s">
+      <c r="L4" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="O4" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="P4" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="Q4" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="K4" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="L4" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="M4" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="O4" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="P4" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="Q4" s="6" t="s">
-        <v>214</v>
-      </c>
       <c r="R4" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="S4" s="6" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="T4" s="6" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
       <c r="U4" s="6" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" s="6" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" s="6" customFormat="1" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>21</v>
       </c>
@@ -2081,176 +2204,176 @@
         <v>22</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="I5" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>44</v>
-      </c>
       <c r="L5" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="N5" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="O5" s="6" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="P5" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="Q5" s="6" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="S5" s="6" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="T5" s="6" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="U5" s="6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" s="6" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="I6" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="J6" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="K6" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="J6" s="6" t="s">
+      <c r="L6" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="N6" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="O6" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="P6" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q6" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="R6" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="T6" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="U6" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="K6" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="L6" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="M6" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="O6" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="P6" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="Q6" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="R6" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="S6" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="T6" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="U6" s="6" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:21" s="6" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>22</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="I7" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="K7" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>56</v>
-      </c>
       <c r="L7" s="6" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="N7" s="6" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="O7" s="6" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="P7" s="6" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" s="6" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>21</v>
       </c>
@@ -2258,58 +2381,58 @@
         <v>22</v>
       </c>
       <c r="C8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="J8" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="K8" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>62</v>
-      </c>
       <c r="L8" s="6" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="N8" s="6" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="O8" s="6" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="P8" s="6" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="Q8" s="6" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="S8" s="6" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="T8" s="6" t="s">
-        <v>208</v>
+        <v>199</v>
       </c>
       <c r="U8" s="6" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" s="6" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
@@ -2317,114 +2440,114 @@
         <v>22</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="J9" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="K9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="K9" s="6" t="s">
-        <v>69</v>
-      </c>
       <c r="L9" s="6" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="M9" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="N9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="O9" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="P9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q9" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="S9" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="T9" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="U9" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" s="6" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="J10" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="K10" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="N9" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="O9" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="P9" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q9" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="R9" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="S9" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="T9" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="U9" s="6" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" s="6" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>265</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>266</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="L10" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="M10" s="13" t="s">
-        <v>172</v>
-      </c>
-      <c r="N10" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="O10" s="13" t="s">
-        <v>262</v>
+      <c r="L10" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="M10" s="14" t="s">
+        <v>277</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>275</v>
+      </c>
+      <c r="O10" s="14" t="s">
+        <v>278</v>
       </c>
       <c r="P10" s="13" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="Q10" s="13" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="R10" s="13" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="S10" s="13" t="s">
-        <v>264</v>
-      </c>
-      <c r="T10" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="U10" s="13" t="s">
-        <v>174</v>
+        <v>253</v>
+      </c>
+      <c r="T10" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="U10" s="14" t="s">
+        <v>276</v>
       </c>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2435,58 +2558,58 @@
         <v>22</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="K11" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>75</v>
-      </c>
       <c r="L11" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="M11" s="6" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="N11" s="6" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="O11" s="6" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="P11" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="Q11" s="6" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="S11" s="6" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="T11" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="U11" s="6" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" s="6" customFormat="1" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" s="6" customFormat="1" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>21</v>
       </c>
@@ -2494,55 +2617,55 @@
         <v>22</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="K12" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>81</v>
-      </c>
       <c r="L12" s="6" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="M12" s="6" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="N12" s="6" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="O12" s="6" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="Q12" s="6" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="S12" s="6" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="T12" s="6" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="U12" s="6" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" spans="1:21" s="6" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2553,55 +2676,55 @@
         <v>22</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>85</v>
+        <v>290</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>86</v>
+        <v>291</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="L13" s="6" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="N13" s="6" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="O13" s="6" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="P13" s="6" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="Q13" s="6" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="S13" s="6" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="T13" s="6" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="U13" s="6" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
     </row>
     <row r="14" spans="1:21" s="6" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2612,55 +2735,55 @@
         <v>22</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="J14" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="K14" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="L14" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="M14" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="N14" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="O14" s="6" t="s">
         <v>238</v>
       </c>
-      <c r="K14" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="L14" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="M14" s="6" t="s">
+      <c r="P14" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q14" s="6" t="s">
         <v>239</v>
       </c>
-      <c r="N14" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="O14" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="P14" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="Q14" s="6" t="s">
-        <v>248</v>
-      </c>
       <c r="R14" s="6" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
       <c r="S14" s="6" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
       <c r="T14" s="6" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="U14" s="6" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
     </row>
     <row r="15" spans="1:21" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -2671,57 +2794,57 @@
         <v>22</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="F15" s="6"/>
       <c r="G15" s="6"/>
       <c r="H15" s="6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="L15" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>28</v>
+        <v>265</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="N15" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="O15" s="6" t="s">
+        <v>280</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S15" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="T15" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="U15" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="U15" s="6" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
@@ -2729,55 +2852,55 @@
         <v>21</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>253</v>
+        <v>282</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>256</v>
+        <v>283</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="P16" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="Q16" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="R16" s="6" t="s">
-        <v>260</v>
-      </c>
-      <c r="S16" s="6" t="s">
-        <v>261</v>
+        <v>248</v>
+      </c>
+      <c r="P16" s="13" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q16" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="R16" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="S16" s="13" t="s">
+        <v>251</v>
       </c>
       <c r="T16" s="6" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
       <c r="U16" s="6" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2785,55 +2908,55 @@
         <v>21</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F17" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>106</v>
-      </c>
       <c r="H17" s="6" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="L17" s="6" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="M17" s="6" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="N17" s="6" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="O17" s="6" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="P17" s="6" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="Q17" s="6" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="R17" s="6" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="S17" s="6" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="T17" s="6" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="U17" s="6" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:21" s="6" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2841,55 +2964,55 @@
         <v>21</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="L18" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="M18" s="6" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>192</v>
+        <v>183</v>
       </c>
       <c r="P18" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="Q18" s="6" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
       <c r="R18" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="S18" s="6" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="T18" s="6" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="U18" s="6" t="s">
-        <v>193</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:21" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -2897,55 +3020,55 @@
         <v>21</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>196</v>
+        <v>187</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="O19" s="6" t="s">
-        <v>197</v>
+        <v>188</v>
       </c>
       <c r="P19" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="Q19" s="6" t="s">
-        <v>198</v>
+        <v>189</v>
       </c>
       <c r="R19" s="6" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="S19" s="6" t="s">
-        <v>199</v>
+        <v>190</v>
       </c>
       <c r="T19" s="6" t="s">
-        <v>195</v>
+        <v>186</v>
       </c>
       <c r="U19" s="6" t="s">
-        <v>200</v>
+        <v>191</v>
       </c>
     </row>
     <row r="20" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
@@ -2953,55 +3076,55 @@
         <v>21</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>201</v>
+        <v>192</v>
       </c>
       <c r="M20" s="6" t="s">
-        <v>202</v>
+        <v>193</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="Q20" s="6" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
       <c r="R20" s="6" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
       <c r="S20" s="6" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
       <c r="T20" s="6" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="U20" s="6" t="s">
-        <v>204</v>
+        <v>195</v>
       </c>
     </row>
     <row r="21" spans="1:21" ht="78.75" x14ac:dyDescent="0.25">
@@ -3009,68 +3132,68 @@
         <v>21</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="G21" s="6" t="s">
         <v>21</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="L21" s="10" t="s">
-        <v>166</v>
-      </c>
-      <c r="M21" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="N21" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="O21" s="10" t="s">
-        <v>28</v>
+        <v>267</v>
+      </c>
+      <c r="L21" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="N21" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="O21" s="6" t="s">
+        <v>287</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="Q21" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="R21" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="S21" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="T21" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="U21" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="U21" s="6" t="s">
+        <v>289</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:U21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="5" type="noConversion"/>
-  <dataValidations count="2">
+  <dataValidations disablePrompts="1" count="2">
     <dataValidation type="list" allowBlank="1" sqref="A2:A200 G2:G200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"是,否"</formula1>
     </dataValidation>
@@ -3096,13 +3219,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -3113,7 +3236,7 @@
         <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -3121,10 +3244,10 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -3135,7 +3258,7 @@
         <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -3143,10 +3266,10 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -3157,7 +3280,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -3165,10 +3288,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="C7" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -3187,47 +3310,47 @@
   <sheetData>
     <row r="1" spans="1:1" ht="21" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="10" spans="1:1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -3247,18 +3370,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="12" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3266,7 +3389,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3274,23 +3397,23 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>143</v>
       </c>
       <c r="B5" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="B6" t="s">
-        <v>153</v>
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: document id-based outfit rules
</commit_message>
<xml_diff>
--- a/data/i18n/dictionary_entries.xlsx
+++ b/data/i18n/dictionary_entries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yezi\G_project\S2_mission_game\fukuchange_v2\data\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34398BC9-FDC8-48A7-8959-8B5EAE34E5DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73371F13-863D-48F8-981A-75D36EDC6728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1965" yWindow="480" windowWidth="17205" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7725" yWindow="150" windowWidth="20700" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="詞典資料" sheetId="1" r:id="rId1"/>
@@ -341,7 +341,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="298">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="295">
   <si>
     <t>啟用</t>
   </si>
@@ -1262,10 +1262,6 @@
   </si>
   <si>
     <t>黑色，是沉穩低調的經典色彩。</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>紫色，是高貴浪漫的迷人色彩。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1378,14 +1374,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>花布仔</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>faˊ bu eˋ</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>藍衫</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1436,7 +1424,7 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>保護膝頭个</t>
+    <t>紫色，是高貴浪漫的迷人色彩。沉穩色調不僅百搭，更是遮髒的好幫手！</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -2041,25 +2029,25 @@
         <v>26</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="J2" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="K2" s="6" t="s">
         <v>268</v>
       </c>
-      <c r="K2" s="6" t="s">
-        <v>269</v>
-      </c>
       <c r="L2" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="M2" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="N2" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="O2" s="6" t="s">
         <v>273</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="O2" s="6" t="s">
-        <v>274</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>27</v>
@@ -2074,10 +2062,10 @@
         <v>27</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="U2" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2161,7 +2149,7 @@
         <v>35</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>196</v>
@@ -2220,7 +2208,7 @@
         <v>40</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>155</v>
@@ -2338,7 +2326,7 @@
         <v>51</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>198</v>
@@ -2456,7 +2444,7 @@
         <v>62</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>63</v>
@@ -2527,13 +2515,13 @@
         <v>163</v>
       </c>
       <c r="M10" s="14" t="s">
+        <v>276</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>274</v>
+      </c>
+      <c r="O10" s="14" t="s">
         <v>277</v>
-      </c>
-      <c r="N10" s="14" t="s">
-        <v>275</v>
-      </c>
-      <c r="O10" s="14" t="s">
-        <v>278</v>
       </c>
       <c r="P10" s="13" t="s">
         <v>163</v>
@@ -2551,7 +2539,7 @@
         <v>163</v>
       </c>
       <c r="U10" s="14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2666,9 +2654,9 @@
         <v>235</v>
       </c>
       <c r="T12" s="14" t="s">
-        <v>297</v>
-      </c>
-      <c r="U12" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="U12" s="14" t="s">
         <v>228</v>
       </c>
     </row>
@@ -2689,10 +2677,10 @@
         <v>79</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>80</v>
@@ -2719,7 +2707,7 @@
         <v>172</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="S13" s="6" t="s">
         <v>173</v>
@@ -2818,19 +2806,19 @@
         <v>245</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="L15" s="6" t="s">
         <v>245</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N15" s="6" t="s">
         <v>245</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>27</v>
@@ -2848,7 +2836,7 @@
         <v>245</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
@@ -2868,7 +2856,7 @@
         <v>95</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>244</v>
@@ -2877,10 +2865,10 @@
         <v>96</v>
       </c>
       <c r="L16" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="M16" s="6" t="s">
         <v>282</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>283</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>247</v>
@@ -3075,7 +3063,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="20" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" s="6" customFormat="1" ht="126" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
@@ -3092,7 +3080,7 @@
         <v>113</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>264</v>
+        <v>294</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>192</v>
@@ -3154,26 +3142,26 @@
         <v>21</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="K21" s="6" t="s">
         <v>266</v>
       </c>
-      <c r="K21" s="6" t="s">
-        <v>267</v>
-      </c>
       <c r="L21" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="M21" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="M21" s="6" t="s">
+      <c r="N21" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="N21" s="6" t="s">
+      <c r="O21" s="6" t="s">
         <v>286</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>287</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>27</v>
@@ -3188,10 +3176,10 @@
         <v>27</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>288</v>
+        <v>265</v>
       </c>
       <c r="U21" s="6" t="s">
-        <v>289</v>
+        <v>266</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: adjust weather and dirty context rules
</commit_message>
<xml_diff>
--- a/data/i18n/dictionary_entries.xlsx
+++ b/data/i18n/dictionary_entries.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yezi\G_project\S2_mission_game\fukuchange_v2\data\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73371F13-863D-48F8-981A-75D36EDC6728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB23E89-F168-41F6-97D3-DBE9B41B124E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7725" yWindow="150" windowWidth="20700" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15000" yWindow="150" windowWidth="13425" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="詞典資料" sheetId="1" r:id="rId1"/>
@@ -1245,10 +1245,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>防水防泥的橡膠中筒雨靴。</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>適合在郊外穿，能遮擋蚊蟲。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1258,10 +1254,6 @@
   </si>
   <si>
     <t>白色，是如雪般潔白的杭菊色彩。</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>黑色，是沉穩低調的經典色彩。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1424,7 +1416,15 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>紫色，是高貴浪漫的迷人色彩。沉穩色調不僅百搭，更是遮髒的好幫手！</t>
+    <t>紫色，是高貴浪漫的迷人色彩。沉穩色調不僅百搭，更是遮髒的顏色之一！</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>黑色，是沉穩低調的經典色彩，也是遮髒的顏色之一！</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>不管哪種顏色，都防水防泥的橡膠中筒雨靴。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -2029,25 +2029,25 @@
         <v>26</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="N2" s="6" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>27</v>
@@ -2062,10 +2062,10 @@
         <v>27</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="U2" s="6" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="3" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -2090,7 +2090,7 @@
         <v>31</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="J3" s="6" t="s">
         <v>147</v>
@@ -2149,7 +2149,7 @@
         <v>35</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>196</v>
@@ -2208,7 +2208,7 @@
         <v>40</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>155</v>
@@ -2326,7 +2326,7 @@
         <v>51</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>198</v>
@@ -2444,7 +2444,7 @@
         <v>62</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>63</v>
@@ -2483,7 +2483,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="10" spans="1:21" s="6" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" s="6" customFormat="1" ht="59.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>211</v>
       </c>
@@ -2503,7 +2503,7 @@
         <v>258</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>259</v>
+        <v>294</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>163</v>
@@ -2515,13 +2515,13 @@
         <v>163</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="N10" s="14" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="O10" s="14" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="P10" s="13" t="s">
         <v>163</v>
@@ -2539,7 +2539,7 @@
         <v>163</v>
       </c>
       <c r="U10" s="14" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2677,10 +2677,10 @@
         <v>79</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>80</v>
@@ -2707,7 +2707,7 @@
         <v>172</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="S13" s="6" t="s">
         <v>173</v>
@@ -2806,19 +2806,19 @@
         <v>245</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="L15" s="6" t="s">
         <v>245</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="N15" s="6" t="s">
         <v>245</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>27</v>
@@ -2836,7 +2836,7 @@
         <v>245</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
@@ -2856,7 +2856,7 @@
         <v>95</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="J16" s="6" t="s">
         <v>244</v>
@@ -2865,10 +2865,10 @@
         <v>96</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>247</v>
@@ -2895,7 +2895,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="17" spans="1:21" s="6" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" s="6" customFormat="1" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>21</v>
       </c>
@@ -2912,7 +2912,7 @@
         <v>99</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="J17" s="6" t="s">
         <v>100</v>
@@ -2951,7 +2951,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:21" s="6" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" s="6" customFormat="1" ht="72.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>21</v>
       </c>
@@ -2968,7 +2968,7 @@
         <v>104</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J18" s="6" t="s">
         <v>181</v>
@@ -3007,7 +3007,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:21" s="6" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" s="6" customFormat="1" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>21</v>
       </c>
@@ -3024,7 +3024,7 @@
         <v>108</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>263</v>
+        <v>293</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>109</v>
@@ -3063,7 +3063,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="20" spans="1:21" s="6" customFormat="1" ht="126" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" s="6" customFormat="1" ht="141.75" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
@@ -3080,7 +3080,7 @@
         <v>113</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>192</v>
@@ -3142,26 +3142,26 @@
         <v>21</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="L21" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="M21" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="N21" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="M21" s="6" t="s">
+      <c r="O21" s="6" t="s">
         <v>284</v>
-      </c>
-      <c r="N21" s="6" t="s">
-        <v>285</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>286</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>27</v>
@@ -3176,10 +3176,10 @@
         <v>27</v>
       </c>
       <c r="T21" s="6" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="U21" s="6" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add 300-round question simulation script and report, update deny_items for stage 6 swimming question
</commit_message>
<xml_diff>
--- a/data/i18n/dictionary_entries.xlsx
+++ b/data/i18n/dictionary_entries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Yezi\G_project\S2_mission_game\fukuchange_v2\data\i18n\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EB23E89-F168-41F6-97D3-DBE9B41B124E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ACE48FC-D6A6-42EB-8E10-C1A4251B349E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="15000" yWindow="150" windowWidth="13425" windowHeight="15225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1281,10 +1281,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>花布，充滿熱情喜慶與傳統風情的花色。</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t>短袖衫</t>
   </si>
   <si>
@@ -1425,6 +1421,10 @@
   </si>
   <si>
     <t>不管哪種顏色，都防水防泥的橡膠中筒雨靴。</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>花布，鮮艷熱情，充滿傳統風情的亮色系圖樣。</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -2029,7 +2029,7 @@
         <v>26</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J2" s="6" t="s">
         <v>265</v>
@@ -2041,13 +2041,13 @@
         <v>265</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="N2" s="6" t="s">
         <v>265</v>
       </c>
       <c r="O2" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P2" s="10" t="s">
         <v>27</v>
@@ -2062,7 +2062,7 @@
         <v>27</v>
       </c>
       <c r="T2" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="U2" s="6" t="s">
         <v>266</v>
@@ -2149,7 +2149,7 @@
         <v>35</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J4" s="6" t="s">
         <v>196</v>
@@ -2208,7 +2208,7 @@
         <v>40</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J5" s="6" t="s">
         <v>155</v>
@@ -2326,7 +2326,7 @@
         <v>51</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J7" s="6" t="s">
         <v>198</v>
@@ -2444,7 +2444,7 @@
         <v>62</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>63</v>
@@ -2503,7 +2503,7 @@
         <v>258</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J10" s="6" t="s">
         <v>163</v>
@@ -2515,13 +2515,13 @@
         <v>163</v>
       </c>
       <c r="M10" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="N10" s="14" t="s">
+        <v>271</v>
+      </c>
+      <c r="O10" s="14" t="s">
         <v>274</v>
-      </c>
-      <c r="N10" s="14" t="s">
-        <v>272</v>
-      </c>
-      <c r="O10" s="14" t="s">
-        <v>275</v>
       </c>
       <c r="P10" s="13" t="s">
         <v>163</v>
@@ -2539,7 +2539,7 @@
         <v>163</v>
       </c>
       <c r="U10" s="14" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11" spans="1:21" s="6" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -2677,10 +2677,10 @@
         <v>79</v>
       </c>
       <c r="H13" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>285</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>286</v>
       </c>
       <c r="J13" s="6" t="s">
         <v>80</v>
@@ -2707,7 +2707,7 @@
         <v>172</v>
       </c>
       <c r="R13" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="S13" s="6" t="s">
         <v>173</v>
@@ -2812,13 +2812,13 @@
         <v>245</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="N15" s="6" t="s">
         <v>245</v>
       </c>
       <c r="O15" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="P15" s="10" t="s">
         <v>27</v>
@@ -2836,7 +2836,7 @@
         <v>245</v>
       </c>
       <c r="U15" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:21" s="6" customFormat="1" ht="63" x14ac:dyDescent="0.25">
@@ -2865,10 +2865,10 @@
         <v>96</v>
       </c>
       <c r="L16" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="M16" s="6" t="s">
         <v>279</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>280</v>
       </c>
       <c r="N16" s="6" t="s">
         <v>247</v>
@@ -3024,7 +3024,7 @@
         <v>108</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J19" s="6" t="s">
         <v>109</v>
@@ -3080,7 +3080,7 @@
         <v>113</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J20" s="6" t="s">
         <v>192</v>
@@ -3119,7 +3119,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>21</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>21</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>268</v>
+        <v>294</v>
       </c>
       <c r="I21" s="6"/>
       <c r="J21" s="6" t="s">
@@ -3152,16 +3152,16 @@
         <v>264</v>
       </c>
       <c r="L21" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="M21" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="M21" s="6" t="s">
+      <c r="N21" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="N21" s="6" t="s">
+      <c r="O21" s="6" t="s">
         <v>283</v>
-      </c>
-      <c r="O21" s="6" t="s">
-        <v>284</v>
       </c>
       <c r="P21" s="10" t="s">
         <v>27</v>

</xml_diff>